<commit_message>
Update artifact identifiers and increase file size limits to 10MB
</commit_message>
<xml_diff>
--- a/backend/artifact-identifier-service/data/artifact_metadata.xlsx
+++ b/backend/artifact-identifier-service/data/artifact_metadata.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="xep7o9pcJzF8T0o9pzksg6YbRJo9Wij4RNQ7nAroI8I="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="MnaTFHPXkeFzOwAy3S8saO4iKNI6lL8EES/sFK2WpKo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="50">
   <si>
     <t>artifact_name</t>
   </si>
@@ -63,15 +63,6 @@
     <t>chopping, steel, wood handle, heavy, sharp, utility</t>
   </si>
   <si>
-    <t>guitar</t>
-  </si>
-  <si>
-    <t>A fretted musical instrument with six strings, played by plucking or strumming.</t>
-  </si>
-  <si>
-    <t>acoustic, strings, wood, melody, music, western</t>
-  </si>
-  <si>
     <t>spoon</t>
   </si>
   <si>
@@ -82,13 +73,106 @@
   </si>
   <si>
     <t>kitchen, cutlery, metal, dining, silverware, utility</t>
+  </si>
+  <si>
+    <t>sickle</t>
+  </si>
+  <si>
+    <t>Tool</t>
+  </si>
+  <si>
+    <t>Curved blade used for harvesting crops and cutting grass</t>
+  </si>
+  <si>
+    <t>sickle,agriculture,blade</t>
+  </si>
+  <si>
+    <t>hoe blade</t>
+  </si>
+  <si>
+    <t>Metal blade attached to a handle for digging and farming</t>
+  </si>
+  <si>
+    <t>hoe,agriculture,tool</t>
+  </si>
+  <si>
+    <t>gourd vessel</t>
+  </si>
+  <si>
+    <t>Dried gourd used as a natural container for water or food</t>
+  </si>
+  <si>
+    <t>gourd,container,natural</t>
+  </si>
+  <si>
+    <t>fire stone</t>
+  </si>
+  <si>
+    <t>Stone used to create sparks for starting fire</t>
+  </si>
+  <si>
+    <t>fire,stone,survival</t>
+  </si>
+  <si>
+    <t>double mortar</t>
+  </si>
+  <si>
+    <t>Grinding tool used for processing grains or herbs</t>
+  </si>
+  <si>
+    <t>mortar,grinding,food</t>
+  </si>
+  <si>
+    <t>coconut shell cup</t>
+  </si>
+  <si>
+    <t>Cup made from coconut shell used for drinking</t>
+  </si>
+  <si>
+    <t>coconut,cup,natural</t>
+  </si>
+  <si>
+    <t>clay pot</t>
+  </si>
+  <si>
+    <t>Pot made of clay used for cooking or storage</t>
+  </si>
+  <si>
+    <t>clay,pot,cooking</t>
+  </si>
+  <si>
+    <t>bummadiya</t>
+  </si>
+  <si>
+    <t>Traditional Vedda tool used for food preparation or storage</t>
+  </si>
+  <si>
+    <t>vedda,tool,traditional</t>
+  </si>
+  <si>
+    <t>betel nut crusher</t>
+  </si>
+  <si>
+    <t>Tool used to crush betel nuts</t>
+  </si>
+  <si>
+    <t>betel,crusher,tool</t>
+  </si>
+  <si>
+    <t>arrow</t>
+  </si>
+  <si>
+    <t>Projectile used with a bow for hunting</t>
+  </si>
+  <si>
+    <t>arrow,hunting,weapon</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="12.0"/>
       <color theme="1"/>
@@ -106,6 +190,20 @@
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -121,12 +219,21 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -408,38 +515,155 @@
         <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="D6" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1"/>
-    <row r="8" ht="15.75" customHeight="1"/>
-    <row r="9" ht="15.75" customHeight="1"/>
-    <row r="10" ht="15.75" customHeight="1"/>
-    <row r="11" ht="15.75" customHeight="1"/>
-    <row r="12" ht="15.75" customHeight="1"/>
-    <row r="13" ht="15.75" customHeight="1"/>
-    <row r="14" ht="15.75" customHeight="1"/>
-    <row r="15" ht="15.75" customHeight="1"/>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
     <row r="16" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
@@ -450,7 +674,9 @@
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="4"/>
+    </row>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1"/>
@@ -1423,7 +1649,6 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>